<commit_message>
Feat: subindo atualizações com testes
</commit_message>
<xml_diff>
--- a/prompts.xlsx
+++ b/prompts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario1\Documents\mestrado\ia\at1-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF76AC5D-E574-4059-A2BA-BAB2A9AF6624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7192AF4C-20E2-4C5B-B3AF-06F9E1D4D8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -126,12 +126,33 @@
   percentual de alternativas selecionadas ou deixadas de ser selecionadas incorretamente)
   rigorosa. </t>
   </si>
+  <si>
+    <t>A correção não está funcionando bem</t>
+  </si>
+  <si>
+    <t>mais ou menos</t>
+  </si>
+  <si>
+    <t>Crie uma opção para gerar um arquivo csv com as respostas da prova</t>
+  </si>
+  <si>
+    <t>O codigo gerado não funcionou</t>
+  </si>
+  <si>
+    <t>Ele gerou o codigo mas não funcionou</t>
+  </si>
+  <si>
+    <t>Corrija a geração das respostas</t>
+  </si>
+  <si>
+    <t>Dessa vez ele corrigiu e funciona de forma correta</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -151,6 +172,12 @@
     <font>
       <b/>
       <i/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <u/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -338,7 +365,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -383,6 +410,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1517,7 +1547,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="44.33203125" style="1" customWidth="1"/>
@@ -1527,7 +1557,7 @@
     <col min="7" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.6" customHeight="1">
+    <row r="1" spans="1:7" ht="27.6" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1536,7 +1566,7 @@
       <c r="D1" s="13"/>
       <c r="E1" s="14"/>
     </row>
-    <row r="2" spans="1:5" ht="20.25" customHeight="1">
+    <row r="2" spans="1:7" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1553,7 +1583,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="105.6">
+    <row r="3" spans="1:7" ht="105.6">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1568,7 +1598,7 @@
       </c>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="1:5" ht="92.4">
+    <row r="4" spans="1:7" ht="92.4">
       <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
@@ -1585,7 +1615,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="184.8">
+    <row r="5" spans="1:7" ht="184.8">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
@@ -1602,7 +1632,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="237.6">
+    <row r="6" spans="1:7" ht="237.6">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1619,7 +1649,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="26.4">
+    <row r="7" spans="1:7" ht="26.4">
       <c r="A7" s="7" t="s">
         <v>22</v>
       </c>
@@ -1636,65 +1666,92 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="224.4">
+    <row r="8" spans="1:7" ht="224.4">
       <c r="A8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="B8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="G8" s="15"/>
+    </row>
+    <row r="9" spans="1:7" ht="26.4">
+      <c r="A9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="26.4">
+      <c r="A10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
     </row>
-    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
     </row>
-    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="14" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>

</xml_diff>

<commit_message>
Feat: subindo para deploy
</commit_message>
<xml_diff>
--- a/prompts.xlsx
+++ b/prompts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario1\Documents\mestrado\ia\at1-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7192AF4C-20E2-4C5B-B3AF-06F9E1D4D8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E84469-F7BD-4ADC-A746-B5714CE5032A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -146,6 +146,13 @@
   </si>
   <si>
     <t>Dessa vez ele corrigiu e funciona de forma correta</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> agora vamos criar os testes,  use a linguagem Gherkin do Cucumber, que deve ser usado para 
+  implementar os testes de aceitação.</t>
+  </si>
+  <si>
+    <t>Criou os testes</t>
   </si>
 </sst>
 </file>
@@ -402,6 +409,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -410,9 +420,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1558,13 +1565,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.6" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:7" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1680,7 +1687,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="9"/>
-      <c r="G8" s="15"/>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="26.4">
       <c r="A9" s="7" t="s">
@@ -1716,12 +1723,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="20.100000000000001" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+    <row r="11" spans="1:7" ht="39.6">
+      <c r="A11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="7"/>

</xml_diff>